<commit_message>
Added Video bulk upload file
</commit_message>
<xml_diff>
--- a/src/main/resources/uploadfiles/NativeBulkUploadTemplate.xlsx
+++ b/src/main/resources/uploadfiles/NativeBulkUploadTemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rsherkar\IdeaProjects\PulsePointNew\src\main\resources\uploadfiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0BF30D3-572A-4AD3-A148-A7F4F38BCBFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2E62D25-186E-4B07-A47C-498953D30FFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -460,9 +460,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -500,7 +500,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>12</v>
       </c>

</xml_diff>